<commit_message>
Update Talkivana publishing schedule matrix
</commit_message>
<xml_diff>
--- a/tracker/publishing_schedule.xlsx
+++ b/tracker/publishing_schedule.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Slot Availability" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Schedule Matrix'!$A$5:$I$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Schedule Matrix'!$A$5:$I$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -541,7 +541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:I13"/>
+  <dimension ref="A2:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -748,7 +748,7 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Scheduled; currently private</t>
+          <t>Published publicly</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr"/>
@@ -848,8 +848,124 @@
       <c r="H13" s="6" t="inlineStr"/>
       <c r="I13" s="6" t="inlineStr"/>
     </row>
+    <row r="14">
+      <c r="A14" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Short 1: German Directions Vocabulary</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Scheduled; currently private</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr"/>
+      <c r="G14" s="6" t="inlineStr"/>
+      <c r="H14" s="6" t="inlineStr"/>
+      <c r="I14" s="6" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Short 2: Daily Routine Vocabulary</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Scheduled; currently private</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr"/>
+      <c r="F15" s="6" t="inlineStr"/>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr"/>
+      <c r="I15" s="6" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Video 1: Asking for Directions in the City</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Scheduled; currently private</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr"/>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr"/>
+      <c r="H16" s="6" t="inlineStr"/>
+      <c r="I16" s="6" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Video 2: Starting the Morning Routine</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Scheduled; currently private</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr"/>
+      <c r="F17" s="6" t="inlineStr"/>
+      <c r="G17" s="6" t="inlineStr"/>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="I17" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A5:I13"/>
+  <autoFilter ref="A5:I17"/>
   <mergeCells count="2">
     <mergeCell ref="A3:I3"/>
     <mergeCell ref="A2:I2"/>
@@ -1021,7 +1137,7 @@
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>Available</t>
+          <t>Short 1: German Directions Vocabulary</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
@@ -1031,7 +1147,7 @@
       </c>
       <c r="E8" s="11" t="inlineStr">
         <is>
-          <t>Available</t>
+          <t>Short 2: Daily Routine Vocabulary</t>
         </is>
       </c>
       <c r="F8" s="11" t="inlineStr">
@@ -1064,7 +1180,7 @@
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>Available</t>
+          <t>Video 1: Asking for Directions in the City</t>
         </is>
       </c>
       <c r="E9" s="11" t="inlineStr">
@@ -1074,7 +1190,7 @@
       </c>
       <c r="F9" s="11" t="inlineStr">
         <is>
-          <t>Available</t>
+          <t>Video 2: Starting the Morning Routine</t>
         </is>
       </c>
       <c r="G9" s="10">

</xml_diff>